<commit_message>
feat: Implement product import rules and validation, enhance product management features
</commit_message>
<xml_diff>
--- a/sample_data/opening_stock.xlsx
+++ b/sample_data/opening_stock.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -440,11 +440,6 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>store_code</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
           <t>quantity</t>
         </is>
       </c>
@@ -455,12 +450,7 @@
           <t>SKU-101</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
+      <c r="B2" s="2" t="n">
         <v>183</v>
       </c>
     </row>
@@ -470,12 +460,7 @@
           <t>SKU-102</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="B3" s="2" t="n">
         <v>48</v>
       </c>
     </row>
@@ -485,12 +470,7 @@
           <t>SKU-103</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="B4" s="2" t="n">
         <v>26</v>
       </c>
     </row>
@@ -500,12 +480,7 @@
           <t>SKU-104</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="B5" s="2" t="n">
         <v>90</v>
       </c>
     </row>
@@ -515,12 +490,7 @@
           <t>SKU-105</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
+      <c r="B6" s="2" t="n">
         <v>82</v>
       </c>
     </row>
@@ -530,12 +500,7 @@
           <t>SKU-106</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="B7" s="2" t="n">
         <v>77</v>
       </c>
     </row>
@@ -545,12 +510,7 @@
           <t>SKU-107</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
+      <c r="B8" s="2" t="n">
         <v>55</v>
       </c>
     </row>
@@ -560,12 +520,7 @@
           <t>SKU-108</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
+      <c r="B9" s="2" t="n">
         <v>46</v>
       </c>
     </row>
@@ -575,12 +530,7 @@
           <t>SKU-109</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
+      <c r="B10" s="2" t="n">
         <v>193</v>
       </c>
     </row>
@@ -590,12 +540,7 @@
           <t>SKU-110</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n">
+      <c r="B11" s="2" t="n">
         <v>159</v>
       </c>
     </row>
@@ -605,12 +550,7 @@
           <t>SKU-111</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
+      <c r="B12" s="2" t="n">
         <v>42</v>
       </c>
     </row>
@@ -620,12 +560,7 @@
           <t>SKU-112</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
+      <c r="B13" s="2" t="n">
         <v>171</v>
       </c>
     </row>
@@ -635,12 +570,7 @@
           <t>SKU-113</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
+      <c r="B14" s="2" t="n">
         <v>128</v>
       </c>
     </row>
@@ -650,12 +580,7 @@
           <t>SKU-114</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>28</v>
       </c>
     </row>
@@ -665,12 +590,7 @@
           <t>SKU-115</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
+      <c r="B16" s="2" t="n">
         <v>27</v>
       </c>
     </row>
@@ -680,12 +600,7 @@
           <t>SKU-116</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>43</v>
       </c>
     </row>
@@ -695,12 +610,7 @@
           <t>SKU-117</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
+      <c r="B18" s="2" t="n">
         <v>75</v>
       </c>
     </row>
@@ -710,12 +620,7 @@
           <t>SKU-118</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
+      <c r="B19" s="2" t="n">
         <v>79</v>
       </c>
     </row>
@@ -725,12 +630,7 @@
           <t>SKU-119</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>149</v>
       </c>
     </row>
@@ -740,12 +640,7 @@
           <t>SKU-120</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>ST001</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
+      <c r="B21" s="2" t="n">
         <v>174</v>
       </c>
     </row>

</xml_diff>